<commit_message>
add script/query to move production for bayer_tmc registration/enrollment and event
</commit_message>
<xml_diff>
--- a/options.xlsx
+++ b/options.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mithilesh Thakur\Desktop\mysql_dhis2_connector_amrti-104\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048B4A43-6936-4AA1-B1BF-3B85CD2D221A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3299F59F-FD65-4C1A-83E9-AC5C7E55661A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$3523</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2364,8 +2367,8 @@
   <dimension ref="A1:B3523"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.453125" customWidth="1"/>
-    <col min="2" max="2" width="17.90625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="40.26953125" customWidth="1"/>
+    <col min="2" max="2" width="21.90625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>